<commit_message>
Update Input data files; add DB_ProductosEspejo.xlsx
DB_ProductosEspejo.xlsx es requerido por el codigo de esta sesion para
mapear items espejo a su grupo. Los demas archivos Input/*.xlsx reflejan
la actualizacion de datos de negocio del corte mas reciente.
</commit_message>
<xml_diff>
--- a/Input/DB_Tiendas.xlsx
+++ b/Input/DB_Tiendas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prestamo\Documents\Isimo\Proyectos\Distribucion de Fruver\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A82921D-939F-4577-820F-4FA37A189351}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{340FB75C-6AC3-4EBF-8BBC-B01C6B41A24E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{0B837EF7-7BAD-C043-BDCC-D80A63680A1A}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$I$95</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$I$94</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="761" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="753" uniqueCount="217">
   <si>
     <t>COD SIESA</t>
   </si>
@@ -603,12 +603,6 @@
   </si>
   <si>
     <t>ISIMO CIUDAD ORIENTAL</t>
-  </si>
-  <si>
-    <t>SD8</t>
-  </si>
-  <si>
-    <t>ISIMO COSTA AZUL</t>
   </si>
   <si>
     <t>SD9</t>
@@ -1070,7 +1064,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC3D23D1-10E0-9A47-AB1D-3A118B1BB2DD}">
-  <dimension ref="A1:I95"/>
+  <dimension ref="A1:I94"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.75" bestFit="1" customWidth="1"/>
@@ -1136,7 +1130,7 @@
         <v>12</v>
       </c>
       <c r="H2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="I2">
         <v>3</v>
@@ -1165,7 +1159,7 @@
         <v>12</v>
       </c>
       <c r="H3" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="I3">
         <v>2</v>
@@ -1194,7 +1188,7 @@
         <v>12</v>
       </c>
       <c r="H4" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="I4">
         <v>5</v>
@@ -1223,7 +1217,7 @@
         <v>12</v>
       </c>
       <c r="H5" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="I5">
         <v>4</v>
@@ -1252,7 +1246,7 @@
         <v>12</v>
       </c>
       <c r="H6" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="I6">
         <v>4</v>
@@ -1281,7 +1275,7 @@
         <v>12</v>
       </c>
       <c r="H7" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="I7">
         <v>3</v>
@@ -1310,7 +1304,7 @@
         <v>12</v>
       </c>
       <c r="H8" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="I8">
         <v>2</v>
@@ -1339,7 +1333,7 @@
         <v>12</v>
       </c>
       <c r="H9" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="I9">
         <v>4</v>
@@ -1368,7 +1362,7 @@
         <v>12</v>
       </c>
       <c r="H10" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="I10">
         <v>3</v>
@@ -1397,7 +1391,7 @@
         <v>12</v>
       </c>
       <c r="H11" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="I11">
         <v>3</v>
@@ -1426,7 +1420,7 @@
         <v>40</v>
       </c>
       <c r="H12" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="I12">
         <v>4</v>
@@ -1455,7 +1449,7 @@
         <v>40</v>
       </c>
       <c r="H13" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="I13">
         <v>3</v>
@@ -1484,7 +1478,7 @@
         <v>40</v>
       </c>
       <c r="H14" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I14">
         <v>2</v>
@@ -1513,7 +1507,7 @@
         <v>40</v>
       </c>
       <c r="H15" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I15">
         <v>2</v>
@@ -1542,7 +1536,7 @@
         <v>12</v>
       </c>
       <c r="H16" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="I16">
         <v>2</v>
@@ -1571,7 +1565,7 @@
         <v>40</v>
       </c>
       <c r="H17" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="I17">
         <v>3</v>
@@ -1600,7 +1594,7 @@
         <v>40</v>
       </c>
       <c r="H18" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="I18">
         <v>2</v>
@@ -1629,7 +1623,7 @@
         <v>40</v>
       </c>
       <c r="H19" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I19">
         <v>2</v>
@@ -1658,7 +1652,7 @@
         <v>12</v>
       </c>
       <c r="H20" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I20">
         <v>2</v>
@@ -1687,7 +1681,7 @@
         <v>12</v>
       </c>
       <c r="H21" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="I21">
         <v>3</v>
@@ -1716,7 +1710,7 @@
         <v>12</v>
       </c>
       <c r="H22" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="I22">
         <v>3</v>
@@ -1745,7 +1739,7 @@
         <v>12</v>
       </c>
       <c r="H23" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="I23">
         <v>4</v>
@@ -1774,7 +1768,7 @@
         <v>12</v>
       </c>
       <c r="H24" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="I24">
         <v>3</v>
@@ -1803,7 +1797,7 @@
         <v>40</v>
       </c>
       <c r="H25" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="I25">
         <v>3</v>
@@ -1832,7 +1826,7 @@
         <v>12</v>
       </c>
       <c r="H26" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="I26">
         <v>2</v>
@@ -1861,7 +1855,7 @@
         <v>12</v>
       </c>
       <c r="H27" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="I27">
         <v>3</v>
@@ -1890,7 +1884,7 @@
         <v>40</v>
       </c>
       <c r="H28" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="I28">
         <v>2</v>
@@ -1919,7 +1913,7 @@
         <v>12</v>
       </c>
       <c r="H29" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="I29">
         <v>3</v>
@@ -1948,7 +1942,7 @@
         <v>12</v>
       </c>
       <c r="H30" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="I30">
         <v>3</v>
@@ -1977,7 +1971,7 @@
         <v>12</v>
       </c>
       <c r="H31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="I31">
         <v>5</v>
@@ -2006,7 +2000,7 @@
         <v>12</v>
       </c>
       <c r="H32" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="I32">
         <v>2</v>
@@ -2035,7 +2029,7 @@
         <v>40</v>
       </c>
       <c r="H33" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="I33">
         <v>3</v>
@@ -2064,7 +2058,7 @@
         <v>40</v>
       </c>
       <c r="H34" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="I34">
         <v>2</v>
@@ -2093,7 +2087,7 @@
         <v>12</v>
       </c>
       <c r="H35" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="I35">
         <v>2</v>
@@ -2122,7 +2116,7 @@
         <v>40</v>
       </c>
       <c r="H36" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="I36">
         <v>2</v>
@@ -2151,7 +2145,7 @@
         <v>12</v>
       </c>
       <c r="H37" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="I37">
         <v>3</v>
@@ -2180,7 +2174,7 @@
         <v>12</v>
       </c>
       <c r="H38" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I38">
         <v>2</v>
@@ -2209,7 +2203,7 @@
         <v>12</v>
       </c>
       <c r="H39" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="I39">
         <v>3</v>
@@ -2238,7 +2232,7 @@
         <v>12</v>
       </c>
       <c r="H40" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="I40">
         <v>3</v>
@@ -2267,7 +2261,7 @@
         <v>12</v>
       </c>
       <c r="H41" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I41">
         <v>2</v>
@@ -2296,7 +2290,7 @@
         <v>12</v>
       </c>
       <c r="H42" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="I42">
         <v>3</v>
@@ -2325,7 +2319,7 @@
         <v>40</v>
       </c>
       <c r="H43" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="I43">
         <v>2</v>
@@ -2354,7 +2348,7 @@
         <v>40</v>
       </c>
       <c r="H44" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="I44">
         <v>2</v>
@@ -2383,7 +2377,7 @@
         <v>12</v>
       </c>
       <c r="H45" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="I45">
         <v>3</v>
@@ -2412,7 +2406,7 @@
         <v>12</v>
       </c>
       <c r="H46" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="I46">
         <v>3</v>
@@ -2441,7 +2435,7 @@
         <v>12</v>
       </c>
       <c r="H47" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="I47">
         <v>4</v>
@@ -2470,7 +2464,7 @@
         <v>40</v>
       </c>
       <c r="H48" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="I48">
         <v>3</v>
@@ -2499,7 +2493,7 @@
         <v>12</v>
       </c>
       <c r="H49" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="I49">
         <v>3</v>
@@ -2528,7 +2522,7 @@
         <v>40</v>
       </c>
       <c r="H50" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="I50">
         <v>2</v>
@@ -2557,7 +2551,7 @@
         <v>40</v>
       </c>
       <c r="H51" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="I51">
         <v>3</v>
@@ -2586,7 +2580,7 @@
         <v>12</v>
       </c>
       <c r="H52" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="I52">
         <v>3</v>
@@ -2615,7 +2609,7 @@
         <v>40</v>
       </c>
       <c r="H53" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I53">
         <v>2</v>
@@ -2644,7 +2638,7 @@
         <v>12</v>
       </c>
       <c r="H54" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="I54">
         <v>3</v>
@@ -2673,7 +2667,7 @@
         <v>12</v>
       </c>
       <c r="H55" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="I55">
         <v>3</v>
@@ -2702,7 +2696,7 @@
         <v>12</v>
       </c>
       <c r="H56" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="I56">
         <v>4</v>
@@ -2731,7 +2725,7 @@
         <v>12</v>
       </c>
       <c r="H57" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="I57">
         <v>2</v>
@@ -2760,7 +2754,7 @@
         <v>12</v>
       </c>
       <c r="H58" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="I58">
         <v>4</v>
@@ -2789,7 +2783,7 @@
         <v>12</v>
       </c>
       <c r="H59" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="I59">
         <v>4</v>
@@ -2818,7 +2812,7 @@
         <v>12</v>
       </c>
       <c r="H60" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="I60">
         <v>4</v>
@@ -2847,7 +2841,7 @@
         <v>12</v>
       </c>
       <c r="H61" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="I61">
         <v>3</v>
@@ -2876,7 +2870,7 @@
         <v>40</v>
       </c>
       <c r="H62" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="I62">
         <v>2</v>
@@ -2905,7 +2899,7 @@
         <v>12</v>
       </c>
       <c r="H63" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="I63">
         <v>2</v>
@@ -2934,7 +2928,7 @@
         <v>12</v>
       </c>
       <c r="H64" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="I64">
         <v>3</v>
@@ -2963,7 +2957,7 @@
         <v>12</v>
       </c>
       <c r="H65" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="I65">
         <v>3</v>
@@ -2992,7 +2986,7 @@
         <v>12</v>
       </c>
       <c r="H66" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="I66">
         <v>3</v>
@@ -3021,7 +3015,7 @@
         <v>12</v>
       </c>
       <c r="H67" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="I67">
         <v>4</v>
@@ -3050,7 +3044,7 @@
         <v>12</v>
       </c>
       <c r="H68" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="I68">
         <v>3</v>
@@ -3079,7 +3073,7 @@
         <v>40</v>
       </c>
       <c r="H69" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="I69">
         <v>2</v>
@@ -3108,7 +3102,7 @@
         <v>12</v>
       </c>
       <c r="H70" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="I70">
         <v>2</v>
@@ -3137,7 +3131,7 @@
         <v>40</v>
       </c>
       <c r="H71" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="I71">
         <v>4</v>
@@ -3166,7 +3160,7 @@
         <v>40</v>
       </c>
       <c r="H72" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="I72">
         <v>3</v>
@@ -3195,7 +3189,7 @@
         <v>40</v>
       </c>
       <c r="H73" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I73">
         <v>2</v>
@@ -3224,7 +3218,7 @@
         <v>40</v>
       </c>
       <c r="H74" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="I74">
         <v>3</v>
@@ -3253,7 +3247,7 @@
         <v>12</v>
       </c>
       <c r="H75" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="I75">
         <v>3</v>
@@ -3282,7 +3276,7 @@
         <v>40</v>
       </c>
       <c r="H76" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="I76">
         <v>2</v>
@@ -3311,7 +3305,7 @@
         <v>40</v>
       </c>
       <c r="H77" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="I77">
         <v>2</v>
@@ -3340,7 +3334,7 @@
         <v>12</v>
       </c>
       <c r="H78" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="I78">
         <v>2</v>
@@ -3369,7 +3363,7 @@
         <v>40</v>
       </c>
       <c r="H79" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="I79">
         <v>3</v>
@@ -3398,7 +3392,7 @@
         <v>12</v>
       </c>
       <c r="H80" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="I80">
         <v>2</v>
@@ -3427,7 +3421,7 @@
         <v>40</v>
       </c>
       <c r="H81" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I81">
         <v>2</v>
@@ -3456,7 +3450,7 @@
         <v>12</v>
       </c>
       <c r="H82" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="I82">
         <v>2</v>
@@ -3485,7 +3479,7 @@
         <v>12</v>
       </c>
       <c r="H83" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="I83">
         <v>3</v>
@@ -3514,7 +3508,7 @@
         <v>40</v>
       </c>
       <c r="H84" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="I84">
         <v>3</v>
@@ -3540,13 +3534,13 @@
         <v>15</v>
       </c>
       <c r="G85" t="s">
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="H85" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="I85">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
@@ -3557,7 +3551,7 @@
         <v>190</v>
       </c>
       <c r="C86" t="s">
-        <v>11</v>
+        <v>45</v>
       </c>
       <c r="D86" t="s">
         <v>13</v>
@@ -3566,13 +3560,13 @@
         <v>14</v>
       </c>
       <c r="F86" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="G86" t="s">
         <v>12</v>
       </c>
       <c r="H86" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="I86">
         <v>2</v>
@@ -3595,16 +3589,16 @@
         <v>14</v>
       </c>
       <c r="F87" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="G87" t="s">
         <v>12</v>
       </c>
       <c r="H87" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="I87">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
@@ -3624,13 +3618,13 @@
         <v>14</v>
       </c>
       <c r="F88" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="G88" t="s">
         <v>12</v>
       </c>
       <c r="H88" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="I88">
         <v>3</v>
@@ -3653,16 +3647,16 @@
         <v>14</v>
       </c>
       <c r="F89" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="G89" t="s">
         <v>12</v>
       </c>
       <c r="H89" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="I89">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
@@ -3673,7 +3667,7 @@
         <v>198</v>
       </c>
       <c r="C90" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="D90" t="s">
         <v>13</v>
@@ -3682,13 +3676,13 @@
         <v>14</v>
       </c>
       <c r="F90" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="G90" t="s">
         <v>12</v>
       </c>
       <c r="H90" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="I90">
         <v>2</v>
@@ -3702,7 +3696,7 @@
         <v>200</v>
       </c>
       <c r="C91" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="D91" t="s">
         <v>13</v>
@@ -3711,7 +3705,7 @@
         <v>14</v>
       </c>
       <c r="F91" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G91" t="s">
         <v>12</v>
@@ -3746,7 +3740,7 @@
         <v>12</v>
       </c>
       <c r="H92" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="I92">
         <v>2</v>
@@ -3760,7 +3754,7 @@
         <v>204</v>
       </c>
       <c r="C93" t="s">
-        <v>45</v>
+        <v>11</v>
       </c>
       <c r="D93" t="s">
         <v>13</v>
@@ -3769,13 +3763,13 @@
         <v>14</v>
       </c>
       <c r="F93" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="G93" t="s">
         <v>12</v>
       </c>
       <c r="H93" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="I93">
         <v>2</v>
@@ -3789,7 +3783,7 @@
         <v>206</v>
       </c>
       <c r="C94" t="s">
-        <v>11</v>
+        <v>35</v>
       </c>
       <c r="D94" t="s">
         <v>13</v>
@@ -3798,49 +3792,19 @@
         <v>14</v>
       </c>
       <c r="F94" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G94" t="s">
         <v>12</v>
       </c>
       <c r="H94" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="I94">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="95" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A95" t="s">
-        <v>207</v>
-      </c>
-      <c r="B95" t="s">
-        <v>208</v>
-      </c>
-      <c r="C95" t="s">
-        <v>35</v>
-      </c>
-      <c r="D95" t="s">
-        <v>13</v>
-      </c>
-      <c r="E95" t="s">
-        <v>14</v>
-      </c>
-      <c r="F95" t="s">
-        <v>18</v>
-      </c>
-      <c r="G95" t="s">
-        <v>12</v>
-      </c>
-      <c r="H95" t="s">
-        <v>215</v>
-      </c>
-      <c r="I95">
         <v>3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I95" xr:uid="{FC3D23D1-10E0-9A47-AB1D-3A118B1BB2DD}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>